<commit_message>
Update Transportation section (final)
</commit_message>
<xml_diff>
--- a/docs/transportation/data/conflicts_log.xlsx
+++ b/docs/transportation/data/conflicts_log.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Conflicts'!$A$1:$H$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Conflicts'!$A$1:$H$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -510,7 +510,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>What this file is</t>
@@ -518,7 +518,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>One row per place where two documents (or two parts of one document) give different facts, dates or numbers. 50 rows: 44 conflicts, 4 reconciled, 1 stale, 1 version.</t>
+          <t>One row per place where two documents (or two parts of one document) give different facts, dates or numbers. 32 rows. Each row names both documents, their dates and the page, slide or section, so that each can be checked.</t>
         </is>
       </c>
     </row>
@@ -530,146 +530,134 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>id; type; topic; document_a; says_a; document_b; says_b; how_to_resolve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
+          <t>id; group; topic; document_a_says; document_a_reference; document_b_says; document_b_reference; note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>type values</t>
+          <t>How to use on the website</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>conflict = the documents disagree and it is not explained. reconciled = looks like a disagreement but is a difference in scope, date or definition. stale = an older public page not updated after a later decision. version = several versions of one document.</t>
+          <t>Report what each document says, with its name, date and page. Do not say which is right unless the note explains the difference. Do not describe intent. Use 'the documents show'.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>How to use on the website</t>
+          <t>What this file does not claim</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Report what each document says, with its name and date. Do not say which is right unless the log says reconciled. Do not describe intent. Use 'the documents show'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+          <t>A row is not a finding of error or wrongdoing. Many rows are ordinary differences between dates, definitions or study areas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>What this file does not claim</t>
+          <t>Where the documents are</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>A row is not a finding of error or wrongdoing. Many rows are ordinary differences between dates, definitions or study areas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+          <t>City Council documents are on the City's council portal (elcerritoca.portal.civicclerk.com); other links are on the website page 'Where City Documents Disagree'. State agreements, the May 18, 2026 letter, the May 19-20, 2026 emails and the Round 9 application are copies from the City or the state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Cautions</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Document names and locators are in the report (sections 5, 7 and 13). City links must be opened in a browser.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Cautions</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>The AHSC agreements were read from scans. Check the page before quoting a number.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1"/>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+          <t>The AHSC agreements and the Round 9 excerpt were read from scans. Check the page before quoting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1"/>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Evidence tags</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Primary document or official agency page read in this project: agenda bills, minutes, resolutions, SGC/HCD/CTC/MTC/BART/CTCAC documents, city plans and reports, the AHSC letter, email chain, Round 9 narrative excerpt, and the AHSC Standard and Disbursement Agreements (scans read by OCR with key pages checked by eye).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>P-proj</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Primary document or official agency page read in this project: agenda bills, minutes, resolutions, SGC/HCD/CTC/MTC/BART/CTCAC documents, city plans and reports, the AHSC letter, email chain, Round 9 narrative excerpt, and the AHSC Standard and Disbursement Agreements (scans read by OCR with key pages checked by eye).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>Primary document from Ira's project files (FY2026-27/28 proposed budget, 2025 agenda bills, resolutions).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>P-proj</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Primary document from Ira's project files (FY2026-27/28 proposed budget, 2025 agenda bills, resolutions).</t>
+          <t>News, advocacy, blog or developer page. Corroboration only.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>CG</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>News, advocacy, blog or developer page. Corroboration only.</t>
+          <t>From the earlier ChatGPT handoff. Not re-checked.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>CG</t>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>From the earlier ChatGPT handoff. Not re-checked.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
           <t>Do not publish as fact.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1"/>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="18" ht="15" customHeight="1"/>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Data sheet</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>The sheet named 'Conflicts' holds the data, header in row 1, one record per row. Companion CSV: conflicts_log.csv (plain numbers, no $ symbols).</t>
         </is>
@@ -686,15 +674,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="36.9" customWidth="1" min="3" max="3"/>
+    <col width="30.6" customWidth="1" min="2" max="2"/>
+    <col width="58.5" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="54.9" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
@@ -707,7 +695,7 @@
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>group</t>
         </is>
       </c>
       <c r="C1" s="7" t="inlineStr">
@@ -717,27 +705,27 @@
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>document_a</t>
+          <t>document_a_says</t>
         </is>
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>says_a</t>
+          <t>document_a_reference</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>document_b</t>
+          <t>document_b_says</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">
         <is>
-          <t>says_b</t>
+          <t>document_b_reference</t>
         </is>
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
-          <t>how_to_resolve</t>
+          <t>note</t>
         </is>
       </c>
     </row>
@@ -749,37 +737,37 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Inclusionary threshold</t>
+          <t>Homes built</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>SPASP web page pp.4-5</t>
+          <t>464 homes and 65,000 sq ft of commercial space finished on 7 sites, 2019 to 2025</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>9+ rental, 10+ for-sale units</t>
+          <t>City of El Cerrito, Economic Development web page, statement on housing and commercial space completed</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Housing deck slide 13</t>
+          <t>"Delivered 400 market rate, affordable and mixed-use housing units" since the Specific Plan was adopted in 2014</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Rental min 10 units; for-sale min 9</t>
+          <t>Strategic Economics, Implementation Strategy for the San Pablo Avenue Specific Plan, July 7, 2026, slide 10</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Ordinance text</t>
+          <t>The 464 figure is for 2019 to 2025 only; the 400 figure covers the longer period since 2014.</t>
         </is>
       </c>
     </row>
@@ -791,39 +779,35 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>SPASP goals</t>
+          <t>Inclusionary housing threshold</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>SPASP web page p.5</t>
+          <t>9 or more rental units and 10 or more for-sale units</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>'six goals' but lists five (2014 list)</t>
+          <t>City of El Cerrito, San Pablo Avenue Specific Plan web page (printed copy), pages 4 and 5</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Implementation deck slide 5; SPASP Ch.1 (redline)</t>
+          <t>Rental projects: minimum project size 10 units. For-sale projects: minimum project size 9 units</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>2022 update has four goals (Enliven San Pablo Avenue; Practical and Market Friendly Development; Support Climate Action Goals; Housing for a Diverse Population). Ch.1 also still contains the 2014 goals A-E</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Read Ch.1 pp.1-18 to 1-20 visually; state both lists with years</t>
-        </is>
-      </c>
+          <t>Strategic Economics, Affordable Housing and Anti-Displacement Strategy, July 7, 2026, slide 13</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -833,39 +817,35 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Priority Development Areas</t>
+          <t>Specific Plan goals</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>SPASP web page p.4</t>
+          <t>"Six goals" identified in the Plan, but the page lists five (Goals A to E)</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>'identifies three PDAs' (Downtown, Midtown, Uptown)</t>
+          <t>City of El Cerrito, San Pablo Avenue Specific Plan web page (printed copy), page 5</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>SPASP Ch.1 sec.1.03.01</t>
+          <t>The 2014 plan has five goals (A to E); the 2022 update has four goals</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>One resolution in 2007 designated San Pablo Avenue as one Mixed-use Corridor PDA; Downtown/Midtown/Uptown are focus areas</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>ABAG/MTC PDA list</t>
-        </is>
-      </c>
+          <t>San Pablo Avenue Specific Plan Update, Chapter 1: Introduction, October 13, 2022 version, PDF pages 32 and 33</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -875,39 +855,35 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Chronology of Housing Element</t>
+          <t>Priority Development Areas</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>SPASP web page p.4</t>
+          <t>The Specific Plan "identifies three Priority Development Areas"</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Plan adopted 2014 'to advance the goals of the 2023-2031 Housing Element'</t>
+          <t>City of El Cerrito, San Pablo Avenue Specific Plan web page (printed copy), page 4</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>SPASP Ch.1; Agenda Bill 6.D</t>
+          <t>City Council and the Association of Bay Area Governments designated San Pablo Avenue as one Mixed-use Corridor PDA in 2007</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>2015 element adopted April 2015 / certified May 2015; 2023-31 element adopted August 15, 2023, certified August 22, 2023</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>Do not repeat the page's wording</t>
-        </is>
-      </c>
+          <t>San Pablo Avenue Specific Plan Update, Chapter 1: Introduction, October 13, 2022 version, PDF page 9</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -917,39 +893,35 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Housing delivered</t>
+          <t>Housing Element the plan advances</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Econ Dev page</t>
+          <t>The Specific Plan was adopted in 2014 "to advance the goals of the City's 2023-2031 Housing Element"</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>464 units and 65,000 sq ft completed on 7 sites, 2019-2025</t>
+          <t>City of El Cerrito, San Pablo Avenue Specific Plan web page (printed copy), page 4</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Implementation deck slide 10; slide 11</t>
+          <t>The Housing Element in place in 2014 and 2015 was adopted in April 2015 and certified in May 2015; the 2023-2031 element was adopted August 15, 2023 and certified August 22, 2023</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>'400 units since 2014'; projects on slide 11 sum to 321 completed + 70 under construction</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>Major Projects list (elcerrito.gov/198/New-Development)</t>
-        </is>
-      </c>
+          <t>San Pablo Avenue Specific Plan Update, Chapter 1: Introduction, October 13, 2022 version, PDF page 4; City Council Agenda Bill, Item 6.D, General Plan Annual Progress Report, March 17, 2026, page 2</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -959,39 +931,35 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Units entitled</t>
+          <t>Hana Gardens</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Implementation deck slide 4</t>
+          <t>63 units</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>1,500 units entitled 'by 2018'</t>
+          <t>Strategic Economics, Affordable Housing and Anti-Displacement Strategy, July 7, 2026, slide 11</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>SPASP Ch.1 Background</t>
+          <t>62 units, "successfully completed in 2018" (bill); 62 units, year built 2019 (report)</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>'As of 2022, over 1,500 housing units and over 122,000 sq ft entitled'</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Ask staff for entitlement dates</t>
-        </is>
-      </c>
+          <t>City Council Agenda Bill, Item 9.C, May 6, 2025 (AHSC application, Parcel C East), page 2; City of El Cerrito, Housing Successor Annual Report for Fiscal Year 2024/2025, Attachment 3 to Agenda Item 6.D, March 17, 2026, page 8</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1001,7 +969,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -1011,29 +979,25 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Housing deck slide 11</t>
+          <t>1715 Elm Street, 16 units (2 restricted), "Outside Plan Area"</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>1715 Elm St: 16 units (2 restricted), outside Plan Area</t>
+          <t>Strategic Economics, Affordable Housing and Anti-Displacement Strategy, July 7, 2026, slide 11</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Implementation deck slide 11; Housing Element progress report</t>
+          <t>1717 Elm Street, 14 units (2 BMR), completed Fall 2025, listed among "Projects in the Plan Area"</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>1717 Elm St: 14 units (2 BMR), completed fall 2025, in Plan Area</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Permit records; two buildings or one?</t>
-        </is>
-      </c>
+          <t>Strategic Economics, Implementation Strategy for the San Pablo Avenue Specific Plan, July 7, 2026, slide 11</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1043,39 +1007,35 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Hana Gardens</t>
+          <t>Address of the second Plaza building</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Housing deck slide 11</t>
+          <t>6617 Fairmount Avenue</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>63 units</t>
+          <t>City Council Agenda Bill, Item 9.C, May 6, 2025 (AHSC application, Parcel C East), page 1</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>SB341 report p.8; May 6, 2025 agenda bill</t>
+          <t>6671 Fairmount Avenue</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>62 units; built 2019 (SB341) vs 'completed in 2018' (bill)</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Regulatory agreement</t>
-        </is>
-      </c>
+          <t>Draft resolution attached to Agenda Bill 9.C, May 6, 2025 (AHSC application, Parcel C East), page 1; City Council Agenda Bill, Item 9.B, May 6, 2025 (predevelopment loan, Parcel C East), page 1; City of El Cerrito, Housing Successor Annual Report for Fiscal Year 2024/2025, Attachment 3 to Agenda Item 6.D, March 17, 2026, page 7</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1085,37 +1045,37 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Parcel C East address</t>
+          <t>del Norte affordable building: Mayfair or Elora</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>May 6, 2025 Agenda Bill 9.C</t>
+          <t>"Mayfair Affordable": a 69-unit affordable housing project that "broke ground in June 2024 and is slated for completion early 2026"</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>6617 Fairmount</t>
+          <t>City Council Agenda Bill, Item 9.C, May 6, 2025 (AHSC application, Parcel C East), pages 2 and 3</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Resolution (same packet); SB341 report</t>
+          <t>"Elora Apartments," 69 affordable units, completed Spring 2026, listed separately from "Mayfair" (156 apartments); the March 17, 2026 bill calls the 69-unit building beside del Norte BART "Elora"</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>6671 Fairmount</t>
+          <t>Strategic Economics, Implementation Strategy for the San Pablo Avenue Specific Plan, July 7, 2026, slide 11; City Council Agenda Bill, Item 6.D, General Plan Annual Progress Report, March 17, 2026, page 3</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Entitlement record</t>
+          <t>The same building appears to be called two different names.</t>
         </is>
       </c>
     </row>
@@ -1127,39 +1087,35 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>reconciled</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>TOD unit counts</t>
+          <t>Climate plan year</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Approval letter (July 3, 2024) p.2</t>
+          <t>"the 2024 Climate Action and Adaptation Plan"</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Master plan = 673 homes, five buildings, excluding Parcel A South</t>
+          <t>City of El Cerrito, Richmond Street Complete Streets project FAQ, printed September 20, 2026, page 10</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>BART; city documents</t>
+          <t>"2023 Climate Action and Adaptation Plan"</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>743 homes, six buildings (= 673 + 70)</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Scope difference, not an error</t>
-        </is>
-      </c>
+          <t>City of El Cerrito, Richmond Street Complete Streets project FAQ, printed September 20, 2026, page 17</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1169,39 +1125,35 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>reconciled</t>
+          <t>Homes, plans and rules</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>'Affordable' in TOD</t>
+          <t>Specific Plan version</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>BART page</t>
+          <t>The page calls the posted text the "adopted 2022 version," with edits shown in red</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>351 affordable of 743 (47%)</t>
+          <t>City of El Cerrito, San Pablo Avenue Specific Plan web page (printed copy), page 1</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Approval letter pp.6-7</t>
+          <t>Page footers of the posted chapters read "August, 2014 - Corrected"</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>163 (30-60% AMI) + 118 (up to 80% AMI) + 70 (Parcel A South) = 351; only 233 at 60% AMI or below</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>State the AMI levels on the website</t>
-        </is>
-      </c>
+          <t>San Pablo Avenue Specific Plan Update, Chapter 1: Introduction, October 13, 2022 version, PDF pages 3 to 10; San Pablo Avenue Specific Plan Update, Chapter 3: Complete Streets, October 13, 2022 version, PDF pages 4 to 11</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1211,37 +1163,37 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Richmond Street traffic volume</t>
+          <t>Richmond Street total cost</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>City FAQ</t>
+          <t>"$11.092 million in funding"</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>8,400 modeled (StreetLight) replaced by 6,400 measured (October 2024)</t>
+          <t>City of El Cerrito, Richmond Street Complete Streets project FAQ, printed September 20, 2026, page 3</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>SGC email May 20, 2026</t>
+          <t>$12,878,610 for all phases, including City administration ($12,798,340 for CCTA activities)</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>'9000 AADT, 25 MPH' used to confirm Class II meets Context Sensitive Bikeway definition</t>
+          <t>City Council Agenda Bill, Item 6.H, Amendment to Cooperative Agreement with the Contra Costa Transportation Authority for the Richmond Street Complete Streets Improvement Project, March 3, 2026, pages 4 and 5</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>Get the AADT source used in the AHSC request</t>
+          <t>The FAQ shows the 2024-25 plan; the March 3, 2026 bill shows the amended plan.</t>
         </is>
       </c>
     </row>
@@ -1253,37 +1205,37 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Richmond Street parking occupancy</t>
+          <t>Richmond Street funding "secured"</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>City FAQ</t>
+          <t>"Secured $9 million from various sources between 2022 and 2024"</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>~46% (October 2024, Richmond St)</t>
+          <t>City Council Study Session presentation, Active Transportation Plan and Complete Streets Policies, July 15, 2025 (Item 9.A), slide 26</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>July 15, 2025 slide 29</t>
+          <t>Funding plan "As of 2023": $10,104,010. "As of 2024-2025": $11,092,010</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>46% (October 2024) and ~33% (May 2025, wider area)</t>
+          <t>City Council Agenda Bill, Item 6.H, Amendment to Cooperative Agreement with the Contra Costa Transportation Authority for the Richmond Street Complete Streets Improvement Project, March 3, 2026, page 5</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Cite both with study area</t>
+          <t>The slide says "secured"; the bill shows the funding plan. The two use different wording.</t>
         </is>
       </c>
     </row>
@@ -1295,39 +1247,35 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Climate plan year</t>
+          <t>Richmond Street total on the state transportation commission form</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Richmond FAQ</t>
+          <t>"Contribution from other sources" $10,836,000, which with the $800,000 allocation is $11,636,000 (my addition)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>'In 2024, the City adopted the CAAP'</t>
+          <t>California Transportation Commission, August 20-21, 2026 meeting, Reference 2.5s.(3), Resolution LPP-A-2627-03, project 2 (Richmond Street), project 2 entry</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Same FAQ</t>
+          <t>Total project cost $12,798,340</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>'2023 Climate Action and Adaptation Plan'</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Adoption resolution</t>
-        </is>
-      </c>
+          <t>City Council Agenda Bill, Item 6.H, Amendment to Cooperative Agreement with the Contra Costa Transportation Authority for the Richmond Street Complete Streets Improvement Project, March 3, 2026, page 5; Exhibit A (Amendment No. 1 to Cooperative Agreement No. 665), attached to Agenda Bill 6.H, March 3, 2026, Attachment B, page 3</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1337,37 +1285,37 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Retail vacancy</t>
+          <t>Richmond Street funding year</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Implementation deck slide 20 text</t>
+          <t>Construction funding "will be included as part of the Fiscal Year 2027-28 budget"</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>~10% (Plan Area context)</t>
+          <t>City Council Agenda Bill, Item 6.H, Amendment to Cooperative Agreement with the Contra Costa Transportation Authority for the Richmond Street Complete Streets Improvement Project, March 3, 2026, page 7</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Same slide chart</t>
+          <t>$4,345,330 shown in FY2027</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>El Cerrito line ~11% (citywide, my reading of the graph)</t>
+          <t>City of El Cerrito, Proposed FY 2026-27 and FY 2027-28 Biennial Budget, pages 417 and 418</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Data appendix</t>
+          <t>FY2027 is the fiscal year that began July 1, 2026.</t>
         </is>
       </c>
     </row>
@@ -1379,39 +1327,35 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Housing Trust Fund</t>
+          <t>Date of the Richmond Street cooperative agreement</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Housing deck slide 15</t>
+          <t>Cooperative Agreement No. 665 entered into "on September 19, 2023"</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>$95,000 remains (July 2026)</t>
+          <t>Resolution attached to Agenda Bill 6.H, March 3, 2026, page 2</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>SB341 report; FY26-27 budget p.134</t>
+          <t>Cooperative Agreement No. 665 entered into "on October 19, 2023"</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>$105,410 cash available at June 30, 2025 of $6,960,307 balance; budget revenue line ~$6.8M</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Budget narrative; balance is mostly receivables</t>
-        </is>
-      </c>
+          <t>Exhibit A (Amendment No. 1 to Cooperative Agreement No. 665), attached to Agenda Bill 6.H, March 3, 2026, page 1</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1421,37 +1365,37 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>$350,000 contributions</t>
+          <t>BART Safe Routes to BART grant for del Norte</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Housing deck slide 15</t>
+          <t>$812,977</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>$350,000 each to Elora and Plaza TOD</t>
+          <t>BART Board memo, Safe Routes to BART Cycle 2 awards, July 31, 2023, revised chart</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>SB341 report</t>
+          <t>$1.5 million</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>$700,000 spent FY2019/20-2023/24 (not split 350/350) plus $350,000 committed May 6, 2025 to Parcel C East</t>
+          <t>BART Safe Routes to BART Cycle 2 fact sheet for El Cerrito del Norte, June 5, 2025, El Cerrito del Norte project entry</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Ask staff which projects received which loans</t>
+          <t>BART's 2023 memo corrects an earlier $1.5 million figure.</t>
         </is>
       </c>
     </row>
@@ -1463,39 +1407,35 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>TOD grant totals</t>
+          <t>Grant funding for the Plaza TOD</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>May 6, 2025 Agenda Bill 9.C</t>
+          <t>The TOD "has cumulatively secured $95 million in grant funding"</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>TOD 'cumulatively secured $95 million in grant funding'</t>
+          <t>City Council Agenda Bill, Item 9.C, May 6, 2025 (AHSC application, Parcel C East), page 2</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Housing deck slide 14; BART October 2025 slide 8</t>
+          <t>The City brought in "over $60 million" to Elora Apartments and the El Cerrito Plaza TOD</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>'over $60 million' for Elora + Plaza; '$50M in transportation infrastructure funding'</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Ask for the list. AHSC R8 + IIGC + CDLAC bond cap = $95.05M, but a bond allocation is not a grant</t>
-        </is>
-      </c>
+          <t>Strategic Economics, Affordable Housing and Anti-Displacement Strategy, July 7, 2026, slide 14</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1505,39 +1445,35 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Measure C wording</t>
+          <t>City housing fund</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Housing deck slide 18</t>
+          <t>"only $95,000 remains" in the City's Affordable Housing Trust Fund</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Parcel tax 'did not pass the necessary voter approval threshold' (in a two-thirds bond context)</t>
+          <t>Strategic Economics, Affordable Housing and Anti-Displacement Strategy, July 7, 2026, slide 15</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>City staff, February 19, 2026 (via news); results</t>
+          <t>$105,410 available cash of a $6,960,307 balance at June 30, 2025</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Simple-majority measure; ~69.7% No unofficial</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Do not reuse the deck wording; get certified results</t>
-        </is>
-      </c>
+          <t>City of El Cerrito, Housing Successor Annual Report for Fiscal Year 2024/2025, Attachment 3 to Agenda Item 6.D, March 17, 2026, pages 4 and 9</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1547,37 +1483,37 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Cooperative agreement date</t>
+          <t>Second Plaza application: City transportation amount</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Resolution (Item 6.H)</t>
+          <t>$2.9 million for the City's sidewalk, crosswalk, pedestrian and bicycle improvements</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Entered September 19, 2023</t>
+          <t>City Council Agenda Bill, Item 9.C, May 6, 2025 (AHSC application, Parcel C East), page 3</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Exhibit A to resolution</t>
+          <t>"$3.5 million for active transportation infrastructure" in the 2025 application</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Entered October 19, 2023</t>
+          <t>City Council Agenda Bill, Item 6.D, General Plan Annual Progress Report, March 17, 2026, page 3</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>CCTA Agreement No. 665</t>
+          <t>The proposed budget also lists $3.5 million under Round 10.</t>
         </is>
       </c>
     </row>
@@ -1589,39 +1525,35 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Budget year for Richmond funding</t>
+          <t>Date of the first Plaza grant agreement</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Agenda Bill 6.H</t>
+          <t>Agreement entered into "on or about October 24, 2025"</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Construction funding 'will be included as part of the FY 2027-28 budget'; construction begins 'next fiscal year'</t>
+          <t>AHSC Round 8 Disbursement Agreement, El Cerrito Plaza Parcel A South, dated for reference November 20, 2025, page 1</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Proposed FY26-27/27-28 budget p.445</t>
+          <t>Signed 10/31/2025 (City and Related) and 11/5/2025 (HCD)</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>$4,345,330 in FY2027 (= FY 2026-27)</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Adopted budget</t>
-        </is>
-      </c>
+          <t>State Standard Agreement No. 24-AHSC-18468 (AHSC Round 8, El Cerrito Plaza Parcel A South), signed October 31 and November 5, 2025, pages 1 and 2</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1631,39 +1563,35 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>reconciled</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Richmond Street funding plans</t>
+          <t>Program Guidelines cited</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Council slide 26 (July 15, 2025)</t>
+          <t>Guidelines "dated October 31, 2019, amended December 9, 2019"</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>'$9 million secured'</t>
+          <t>AHSC Round 8 Disbursement Agreement, El Cerrito Plaza Parcel A South, dated for reference November 20, 2025, page 1</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Item 6.H tables</t>
+          <t>"Round 8 Program Guidelines dated December 14, 2023"; the scoring table says "AHSC Round 7 Guidelines"</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>$10,104,010 (2023); $11,092,010 (2024-25 = FAQ); $12,798,340 (Amendment); $12,878,610 with City admin. CTC form implies $11,636,000</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Cite each with its date</t>
-        </is>
-      </c>
+          <t>State Standard Agreement No. 24-AHSC-18468 (AHSC Round 8, El Cerrito Plaza Parcel A South), signed October 31 and November 5, 2025, pages 3 and 34</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1673,39 +1601,35 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>stale</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Richmond FAQ funding chart</t>
+          <t>Approved date printed on exhibits</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>City FAQ (printed September 20, 2026)</t>
+          <t>"Approved Date: 04/19/2024"</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>$11,092,000 total; AHSC $988,000</t>
+          <t>AHSC Round 8 Disbursement Agreement, El Cerrito Plaza Parcel A South, dated for reference November 20, 2025, exhibit footers, e.g. page 30</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Item 6.H (March 3, 2026; adopted)</t>
+          <t>"Approved Date: 04/11/2024"</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>$12,798,340 plan; AHSC $1,800,600</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>City to update FAQ</t>
-        </is>
-      </c>
+          <t>State Standard Agreement No. 24-AHSC-18468 (AHSC Round 8, El Cerrito Plaza Parcel A South), signed October 31 and November 5, 2025, exhibit footers, e.g. page 3</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1715,39 +1639,35 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>reconciled</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Budget line vs amendment</t>
+          <t>Timing of transportation construction</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>FY26-27 budget p.445</t>
+          <t>"Commencement of construction of STI. 08/01/2026"</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>$4,345,330 city-side line (AHSC $1,800,600; SB1 LPP $800,000; EBMUD-related $1,155,600 + $44,400; Measure A $344,730; SB1 $200,000)</t>
+          <t>State Standard Agreement No. 24-AHSC-18468 (AHSC Round 8, El Cerrito Plaza Parcel A South), signed October 31 and November 5, 2025, page 36</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Amendment No.1</t>
+          <t>Bikeway payments scheduled August 2027 to April 2028</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>$4,795,330 match; difference $450,000 = earlier-year Measure A $300,000 + Measure J $100,000 + SB1 $50,000</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>My arithmetic; fits exactly</t>
-        </is>
-      </c>
+          <t>AHSC Round 8 Disbursement Agreement, El Cerrito Plaza Parcel A South, dated for reference November 20, 2025, page 36, Exhibit D</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -1757,39 +1677,35 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Del Norte cost and OBAG</t>
+          <t>How a scope change is approved</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>WCCTAC September 17, 2021</t>
+          <t>A revision to the STI work "shall require an amendment"; the agreement may not be amended "except in writing executed by all parties"</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Cost $13.25M; OBAG $4.84M</t>
+          <t>State Standard Agreement No. 24-AHSC-18468 (AHSC Round 8, El Cerrito Plaza Parcel A South), signed October 31 and November 5, 2025, page 6, Exhibit A section 3.C; AHSC Round 8 Disbursement Agreement, El Cerrito Plaza Parcel A South, dated for reference November 20, 2025, page 24, section 31</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>BART memo 2023; council slide July 15, 2025; ChatGPT handoff</t>
+          <t>"this email alone can serve as approval"</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>$14.92M (BART); '$12.7M secured' (slide); '$4M OBAG' [CG, unverified]</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>Final cost report</t>
-        </is>
-      </c>
+          <t>Email chain "AHSC Change Request Form Attachment - 24-AHSC-18468," May 19-20, 2026 (4 pages), page 1, May 20, 2026, 2:46 PM</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -1799,39 +1715,35 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>BART SR2B award to Del Norte</t>
+          <t>Bikeway miles</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>BART memo July 31, 2023</t>
+          <t>"The Awarded project had a proposed 2.22 miles of bikeways"</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>$812,977 (corrects earlier $1.5M)</t>
+          <t>Email chain "AHSC Change Request Form Attachment - 24-AHSC-18468," May 19-20, 2026 (4 pages), page 3, May 20, 2026, 9:28 AM</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>BART June 2025 fact sheet</t>
+          <t>"Current Total (A + C): 2.4 lane miles"</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>$1.5 million</t>
-        </is>
-      </c>
-      <c r="H27" s="8" t="inlineStr">
-        <is>
-          <t>BART to correct</t>
-        </is>
-      </c>
+          <t>Email chain "AHSC Change Request Form Attachment - 24-AHSC-18468," May 19-20, 2026 (4 pages), page 2, May 20, 2026, 10:32 AM</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -1841,39 +1753,35 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Del Norte schedule</t>
+          <t>Sidewalk location</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>WCCTAC 2021</t>
+          <t>"Oak Street sidewalks"</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Open to public June 2024</t>
+          <t>State Standard Agreement No. 24-AHSC-18468 (AHSC Round 8, El Cerrito Plaza Parcel A South), signed October 31 and November 5, 2025, page 33; AHSC Round 8 Disbursement Agreement, El Cerrito Plaza Parcel A South, dated for reference November 20, 2025, page 30, Exhibit B</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>City press release; ribbon cutting; FY26-27 budget</t>
+          <t>Heading "Elm/Willow St Sidewalks"</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Groundbreaking March 6, 2024; ribbon cutting July 13, 2026; budget: 'substantially completed', Caltrans final inspection pending</t>
-        </is>
-      </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>Close-out report</t>
-        </is>
-      </c>
+          <t>AHSC Round 8 Disbursement Agreement, El Cerrito Plaza Parcel A South, dated for reference November 20, 2025, page 36, Exhibit D</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -1883,39 +1791,35 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>State grant documents (AHSC)</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Richmond Street walkway length</t>
+          <t>BART railcars in the Round 9 application</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Standard Agreement Ex. E, Provision A-E.7 (p.5 of 17)</t>
+          <t>"two new BART railcars"</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>2,000 linear feet</t>
+          <t>AHSC Round 9 application narrative prompts for El Cerrito Plaza Parcel C East, footer dated March 25, 2025 (excerpt: narrative pages 3, 7, 10, 12, 14, 15), PDF page 1 (narrative page 3)</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>ChatGPT handoff (state award summary)</t>
+          <t>"three new BART railcars"</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>2,350 linear feet [CG, unverified]</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>SGC award summary PDF</t>
-        </is>
-      </c>
+          <t>AHSC Round 9 application narrative prompts for El Cerrito Plaza Parcel C East, footer dated March 25, 2025 (excerpt: narrative pages 3, 7, 10, 12, 14, 15), PDF page 5 (narrative page 14)</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -1925,39 +1829,35 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Richmond Street design and records</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>AHSC Guidelines round</t>
+          <t>Bike lane type on Richmond Street</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Standard Agreement Ex. A sec.1.B</t>
+          <t>"Class IV protected bikeway on Richmond Street" from Moeser Lane to Hill Street</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Round 8 Guidelines (December 14, 2023)</t>
+          <t>AHSC Round 9 application narrative prompts for El Cerrito Plaza Parcel C East, footer dated March 25, 2025 (excerpt: narrative pages 3, 7, 10, 12, 14, 15), PDF page 1 (narrative page 3)</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>Same agreement, Ex. E scoring table</t>
+          <t>"a Class II Bikeway at Richmond Street and at Elm Street from Moeser Lane to Hill Street"; Class IV "does not appear to be a suitable treatment" north of Moeser Lane</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>'AHSC Round 7 Guidelines, Section 107'</t>
-        </is>
-      </c>
-      <c r="H30" s="8" t="inlineStr">
-        <is>
-          <t>HCD</t>
-        </is>
-      </c>
+          <t>City of El Cerrito Public Works Department letter to the California Department of Housing and Community Development, May 18, 2026, page 1; City of El Cerrito, Richmond Street Complete Streets project FAQ, printed September 20, 2026, page 16</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -1967,39 +1867,35 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Richmond Street design and records</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Awarded bikeway miles</t>
+          <t>Richmond Street traffic volume</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>SGC email May 20, 2026</t>
+          <t>October 2024 sensor count: "ADT of 6,400"</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>Awarded project 2.22 miles of bikeways; Lincoln = 1.1</t>
+          <t>City of El Cerrito, Richmond Street Complete Streets project FAQ, printed September 20, 2026, page 8</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>City email May 20, 2026</t>
+          <t>"about 8,400 vehicles daily" (same FAQ); "9000 AADT, 25 MPH" (state email)</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>'Current total' 2.4 lane miles (Lincoln 1.1 + San Diego/Belmont 0.5 + Central 0.8)</t>
-        </is>
-      </c>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>Application screenshot (not shown in the PDF)</t>
-        </is>
-      </c>
+          <t>City of El Cerrito, Richmond Street Complete Streets project FAQ, printed September 20, 2026, page 20; Email chain "AHSC Change Request Form Attachment - 24-AHSC-18468," May 19-20, 2026 (4 pages), page 1, May 20, 2026, 2:46 PM</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -2009,37 +1905,37 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Richmond Street design and records</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>STI milestone vs schedule</t>
+          <t>Agenda item number</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Standard Agreement Ex. E</t>
+          <t>"Agenda Item No. 6.D."</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>STI construction start August 1, 2026</t>
+          <t>City Council Agenda Bill, Item 6.D, General Plan Annual Progress Report, March 17, 2026, page 1</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>Agenda Bill 6.H; FAQ</t>
+          <t>"Agenda Item No. 6.C. Attachment 3"</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>Richmond Street construction 'late Fall 2026'</t>
+          <t>City of El Cerrito, Housing Successor Annual Report for Fiscal Year 2024/2025, Attachment 3 to Agenda Item 6.D, March 17, 2026, page 1</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Any milestone notice or Disbursement Agreement</t>
+          <t>The report is Attachment 3 to the same item.</t>
         </is>
       </c>
     </row>
@@ -2051,798 +1947,38 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>conflict</t>
+          <t>Richmond Street design and records</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Council action July 15, 2025</t>
+          <t>Timing of the consultant's housing analysis</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Richmond Standard (news)</t>
+          <t>The analysis "is on track to be completed in Spring 2026"</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>Council 'approved' the plan</t>
+          <t>Housing Element Annual Progress Report 2025, Attachment 2 to Agenda Item 6.D, March 17, 2026, page 8</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>Agenda bill 9.A; slides 32-33; Item 6.H; FAQ</t>
+          <t>Reports dated July 7, 2026</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Study session; 'No formal action'; council 'affirmed' direction</t>
-        </is>
-      </c>
-      <c r="H33" s="8" t="inlineStr">
-        <is>
-          <t>Minutes for July 15, 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>C33</t>
-        </is>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Richmond Street lane type</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>Richmond Standard</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>'protected' bike lanes</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>CEQA NOE March 20, 2026; FAQ; Item 6.H</t>
-        </is>
-      </c>
-      <c r="G34" s="8" t="inlineStr">
-        <is>
-          <t>Class II buffered/striped bike lanes north of Moeser; Class IV rejected</t>
-        </is>
-      </c>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>Final plans</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>C34</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Round 9 city active-transportation amount</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>May 6, 2025 Agenda Bill 9.C</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>$2.9M (city STI) + $8.9M VTA</t>
-        </is>
-      </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>March 17, 2026 Agenda Bill 6.D; FY26-27 budget</t>
-        </is>
-      </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>$3.5M; budget labels a $3.5M request 'Round 10'</t>
-        </is>
-      </c>
-      <c r="H35" s="8" t="inlineStr">
-        <is>
-          <t>Ira's Round 10 workbook: the $3.5M is the Complete Streets part of a $40.2M Round 10 request. The March 17, 2026 bill's wording about the 2025 application is not explained</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>C35</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Elora vs Mayfair Affordable</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>May 6, 2025 Agenda Bill 9.C</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>'Mayfair Affordable' 69 units by del Norte BART, groundbreaking June 2024, completion early 2026</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>March 17, 2026 Agenda Bill 6.D; decks</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>'Elora' 69 units by del Norte BART, occupancy spring 2026 (11690 San Pablo)</t>
-        </is>
-      </c>
-      <c r="H36" s="8" t="inlineStr">
-        <is>
-          <t>City page elcerrito.gov/1616</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>C36</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>Agenda item number</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Agenda Bill 6.D (March 17, 2026)</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Item 6.D</t>
-        </is>
-      </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>SB341 report footer</t>
-        </is>
-      </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t>'Agenda Item No. 6.C, Attachment 3'</t>
-        </is>
-      </c>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>Clerk</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>C37</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Minutes vs agenda</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Agenda March 3, 2026</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Consent item 6.G (Red Cross proclamation)</t>
-        </is>
-      </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>Minutes March 3, 2026</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>Item 6.G absent; motions cover D-F and A-C, H</t>
-        </is>
-      </c>
-      <c r="H38" s="8" t="inlineStr">
-        <is>
-          <t>Clerk</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>C38</t>
-        </is>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Strategic Economics delivery</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Housing Element progress report</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Analysis 'on track to be completed in Spring 2026'</t>
-        </is>
-      </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>Decks</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="inlineStr">
-        <is>
-          <t>Dated July 7, 2026</t>
-        </is>
-      </c>
-      <c r="H39" s="8" t="inlineStr">
-        <is>
-          <t>Contract scope/schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>C39</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>Parcel A South completion</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>CTCAC report</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Construction September 2025 to January 2027</t>
-        </is>
-      </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>BART</t>
-        </is>
-      </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>Construction began November 2025, about two years</t>
-        </is>
-      </c>
-      <c r="H40" s="8" t="inlineStr">
-        <is>
-          <t>Building permit/inspection status</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>C40</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>SPASP update document version</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>City page</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>'adopted 2022 version' with edits in red; cover/TOC and chapters labeled 10_13_22, cover says October 2022</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>City file name and file metadata</t>
-        </is>
-      </c>
-      <c r="G41" s="8" t="inlineStr">
-        <is>
-          <t>Cover file 'September-2024'; a search result titled it 'December 2022'; Ch.1 metadata 'public review draft 06.14.22'; footers 'August, 2014 - Corrected'; SEIR adopted December 6, 2022</t>
-        </is>
-      </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>Ask clerk/planning for the clean adopted text</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>C41</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>SPASP Chapter 3 vs built Del Norte</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>SPASP Ch.3 secs. 3.03.02.03</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Uptown: bike lanes south of Wall St, Super Sharrows north</t>
-        </is>
-      </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>Del Norte project (2026)</t>
-        </is>
-      </c>
-      <c r="G42" s="8" t="inlineStr">
-        <is>
-          <t>Class IV separated lanes on San Pablo (Knott-Potrero 0.5 mi) and Cutting/Eastshore</t>
-        </is>
-      </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>Visual check of redline pp.3-30 to 3-33</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>C42</t>
-        </is>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>LPP-F money history</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>CTC January 2023 action</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Deleted 'Richmond Street Curb, Signing, Marking' project; $400,000 to Del Norte</t>
-        </is>
-      </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>CTC December 2025 list (Item 6.H Att. 3)</t>
-        </is>
-      </c>
-      <c r="G43" s="8" t="inlineStr">
-        <is>
-          <t>El Cerrito rows show Del Norte $400K and El Dorado-Gladys-B $200K; not Richmond Complete Streets</t>
-        </is>
-      </c>
-      <c r="H43" s="8" t="inlineStr">
-        <is>
-          <t>CTC March 2026 amended list (Ref 4.19)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>C43</t>
-        </is>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement date</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Disbursement Agreement p.1</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement entered into 'on or about October 24, 2025'</t>
-        </is>
-      </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement pp.1-2</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>Signed by the City and Related October 31, 2025 and by HCD November 5, 2025</t>
-        </is>
-      </c>
-      <c r="H44" s="8" t="inlineStr">
-        <is>
-          <t>HCD record of the executed date</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>C44</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>AHSC Guidelines cited</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>Disbursement Agreement p.1</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Guidelines 'dated October 31, 2019, amended December 9, 2019'</t>
-        </is>
-      </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement Ex. A sec.1.B</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="inlineStr">
-        <is>
-          <t>Round 8 Guidelines dated December 14, 2023 (and a 'Round 7' scoring table, see C29)</t>
-        </is>
-      </c>
-      <c r="H45" s="8" t="inlineStr">
-        <is>
-          <t>HCD</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>C45</t>
-        </is>
-      </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>Approved date printed on exhibits</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Disbursement Agreement exhibits</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Approved Date April 19, 2024</t>
-        </is>
-      </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement exhibits</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>Approved Date April 11, 2024</t>
-        </is>
-      </c>
-      <c r="H46" s="8" t="inlineStr">
-        <is>
-          <t>HCD</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>C46</t>
-        </is>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>BART railcars in Round 9 application</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Round 9 narrative, first page of excerpt (narrative p.3)</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>'two new BART railcars'</t>
-        </is>
-      </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>Round 9 narrative, excerpt PDF p.5 (narrative p.14)</t>
-        </is>
-      </c>
-      <c r="G47" s="8" t="inlineStr">
-        <is>
-          <t>'three new BART railcars'</t>
-        </is>
-      </c>
-      <c r="H47" s="8" t="inlineStr">
-        <is>
-          <t>Full application</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>C47</t>
-        </is>
-      </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>Richmond Street bikeway class</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Round 9 application narrative (prompts document dated March 25, 2025)</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Class IV protected bikeway on Richmond Street from Moeser Lane to Hill Street</t>
-        </is>
-      </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>City FAQ; CEQA notice March 20, 2026; May 18, 2026 letter</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t>Class II (buffered/striped) bike lanes; continuous Class IV rejected</t>
-        </is>
-      </c>
-      <c r="H48" s="8" t="inlineStr">
-        <is>
-          <t>Final plans; application scoring sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>C48</t>
-        </is>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>STI #3 sidewalk location</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement Ex. A-E.7; Disbursement Agreement Ex. B</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>'Oak Street sidewalks'</t>
-        </is>
-      </c>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>Disbursement Agreement Ex. D heading</t>
-        </is>
-      </c>
-      <c r="G49" s="8" t="inlineStr">
-        <is>
-          <t>'Elm/Willow St Sidewalks' (heading partly cut)</t>
-        </is>
-      </c>
-      <c r="H49" s="8" t="inlineStr">
-        <is>
-          <t>HCD/City</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>C49</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>STI construction timing</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement Ex. E milestones</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>STI construction start August 1, 2026; completion August 23, 2029</t>
-        </is>
-      </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Disbursement Agreement Ex. D (November 2025)</t>
-        </is>
-      </c>
-      <c r="G50" s="8" t="inlineStr">
-        <is>
-          <t>STI payments scheduled August 2027 to April 2028 (bikeways) and August 2027 to January 2028 (pedestrian)</t>
-        </is>
-      </c>
-      <c r="H50" s="8" t="inlineStr">
-        <is>
-          <t>Milestone notice or amendment</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>C50</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>conflict</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>How an AHSC scope change is approved</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Standard Agreement Ex. A sec.3.C</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Revision to STI work 'shall require an amendment to this Agreement'</t>
-        </is>
-      </c>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>SGC email May 20, 2026; Disbursement Agreement sec.31</t>
-        </is>
-      </c>
-      <c r="G51" s="8" t="inlineStr">
-        <is>
-          <t>'this email alone can serve as approval'; Disbursement Agreement 'shall not be altered or amended except in writing executed by all parties'</t>
-        </is>
-      </c>
-      <c r="H51" s="8" t="inlineStr">
-        <is>
-          <t>HCD</t>
-        </is>
-      </c>
+          <t>Strategic Economics, Implementation Strategy for the San Pablo Avenue Specific Plan, July 7, 2026, cover, slide 1; Strategic Economics, Affordable Housing and Anti-Displacement Strategy, July 7, 2026, cover, slide 1</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H51"/>
+  <autoFilter ref="A1:H33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>